<commit_message>
Add pronghorn public hunt tables
</commit_message>
<xml_diff>
--- a/processed_data/hard_data_exports/hunt_tables/2026/XLXS/2026 MOOSE BULL O.I.L.xlsx
+++ b/processed_data/hard_data_exports/hunt_tables/2026/XLXS/2026 MOOSE BULL O.I.L.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Hunt Table" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hunt Table'!$A$1:$O$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hunt Table'!$A$1:$O$28</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Hunt Table'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -183,8 +183,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="HUNT_TABLE" displayName="HUNT_TABLE" ref="A1:O42" headerRowCount="1">
-  <autoFilter ref="A1:O42"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="HUNT_TABLE" displayName="HUNT_TABLE" ref="A1:O28" headerRowCount="1">
+  <autoFilter ref="A1:O28"/>
   <tableColumns count="15">
     <tableColumn id="1" name="hunt_name"/>
     <tableColumn id="2" name="hunt_code"/>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1549,12 +1549,12 @@
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Bear Springs CWMU</t>
+          <t>Beaver Hollow CWMU</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>MB6200</t>
+          <t>MB6201</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Historical 2025 draw only; season dates not validated in current DATABASE</t>
+          <t>Contact Operator for 2026 season dates</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -1597,37 +1597,21 @@
           <t>1</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>CROSSWALK_CONFIRMED_ACTIVE_SAME_CODE_IN_2025_PDF</t>
-        </is>
-      </c>
-      <c r="L16" s="3" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="M16" s="3" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="3" t="inlineStr"/>
+      <c r="M16" s="3" t="inlineStr"/>
       <c r="N16" s="3" t="inlineStr"/>
-      <c r="O16" s="3" t="inlineStr">
-        <is>
-          <t>4.5</t>
-        </is>
-      </c>
+      <c r="O16" s="3" t="inlineStr"/>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Beaver Hollow CWMU</t>
+          <t>Causey Spring CWMU</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>MB6201</t>
+          <t>MB6202</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -1671,20 +1655,32 @@
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr"/>
-      <c r="L17" s="5" t="inlineStr"/>
-      <c r="M17" s="5" t="inlineStr"/>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
       <c r="N17" s="5" t="inlineStr"/>
-      <c r="O17" s="5" t="inlineStr"/>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Causey Spring CWMU</t>
+          <t>Deseret CWMU</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>MB6202</t>
+          <t>MB6206</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1741,19 +1737,19 @@
       <c r="N18" s="3" t="inlineStr"/>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>3.3</t>
         </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Deseret CWMU</t>
+          <t>East Fork Chalk Creek CWMU</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>MB6206</t>
+          <t>MB6208</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1783,7 +1779,7 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -1793,7 +1789,7 @@
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr"/>
@@ -1810,19 +1806,19 @@
       <c r="N19" s="5" t="inlineStr"/>
       <c r="O19" s="5" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>4.3</t>
         </is>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Durst Mountain CWMU</t>
+          <t>Grass Valley/Clark Canyon CWMU</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>MB6207</t>
+          <t>MB6211</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1847,12 +1843,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Historical 2025 draw only; season dates not validated in current DATABASE</t>
+          <t>Contact Operator for 2026 season dates</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -1862,14 +1858,10 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>CROSSWALK_CONFIRMED_ACTIVE_SAME_CODE_IN_2025_PDF</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="3" t="inlineStr">
         <is>
           <t>2025</t>
@@ -1877,25 +1869,25 @@
       </c>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="N20" s="3" t="inlineStr"/>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>1.8</t>
         </is>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>East Fork Chalk Creek CWMU</t>
+          <t>Skull Crack CWMU</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>MB6208</t>
+          <t>MB6219</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -1952,19 +1944,19 @@
       <c r="N21" s="5" t="inlineStr"/>
       <c r="O21" s="5" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>2.3</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Ensign Ranches CWMU</t>
+          <t>Strawberry Ridge CWMU</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>MB6209</t>
+          <t>MB6222</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1989,7 +1981,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Historical 2025 draw only; season dates not validated in current DATABASE</t>
+          <t>Contact Operator for 2026 season dates</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -2007,11 +1999,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>CROSSWALK_CONFIRMED_ACTIVE_SAME_CODE_IN_2025_PDF</t>
-        </is>
-      </c>
+      <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="3" t="inlineStr">
         <is>
           <t>2025</t>
@@ -2025,19 +2013,19 @@
       <c r="N22" s="3" t="inlineStr"/>
       <c r="O22" s="3" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>2.7</t>
         </is>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Grass Valley/Clark Canyon CWMU</t>
+          <t>Hardscrabble CWMU</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>MB6211</t>
+          <t>MB6251</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -2067,7 +2055,7 @@
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
@@ -2077,7 +2065,7 @@
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr"/>
@@ -2094,19 +2082,19 @@
       <c r="N23" s="5" t="inlineStr"/>
       <c r="O23" s="5" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>5.5</t>
         </is>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Sharp Mountain CWMU</t>
+          <t>Woodruff Creek South CWMU</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>MB6217</t>
+          <t>MB6256</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -2131,7 +2119,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Historical 2025 draw only; season dates not validated in current DATABASE</t>
+          <t>Contact Operator for 2026 season dates</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -2149,11 +2137,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>CROSSWALK_CONFIRMED_ACTIVE_SAME_CODE_IN_2025_PDF</t>
-        </is>
-      </c>
+      <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="3" t="inlineStr">
         <is>
           <t>2025</t>
@@ -2167,19 +2151,19 @@
       <c r="N24" s="3" t="inlineStr"/>
       <c r="O24" s="3" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>4.3</t>
         </is>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Skull Crack CWMU</t>
+          <t>Jacob's Creek CWMU</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>MB6219</t>
+          <t>MB6258</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -2209,7 +2193,7 @@
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -2219,7 +2203,7 @@
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr"/>
@@ -2236,19 +2220,19 @@
       <c r="N25" s="5" t="inlineStr"/>
       <c r="O25" s="5" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.5</t>
         </is>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>South Canyon CWMU</t>
+          <t>Junction Valley CWMU</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>MB6220</t>
+          <t>MB6262</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2273,7 +2257,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Historical 2025 draw only; season dates not validated in current DATABASE</t>
+          <t>Contact Operator for 2026 season dates</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -2291,11 +2275,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>CROSSWALK_CONFIRMED_ACTIVE_SAME_CODE_IN_2025_PDF</t>
-        </is>
-      </c>
+      <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="3" t="inlineStr">
         <is>
           <t>2025</t>
@@ -2309,19 +2289,19 @@
       <c r="N26" s="3" t="inlineStr"/>
       <c r="O26" s="3" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Strawberry Ridge CWMU</t>
+          <t>Little Pole Canyon CWMU</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>MB6222</t>
+          <t>MB6265</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -2365,32 +2345,20 @@
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr"/>
-      <c r="L27" s="5" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="M27" s="5" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
+      <c r="L27" s="5" t="inlineStr"/>
+      <c r="M27" s="5" t="inlineStr"/>
       <c r="N27" s="5" t="inlineStr"/>
-      <c r="O27" s="5" t="inlineStr">
-        <is>
-          <t>2.7</t>
-        </is>
-      </c>
+      <c r="O27" s="5" t="inlineStr"/>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Three C CWMU</t>
+          <t>Weber Florence Creek/Stillman Creek CWMU</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>MB6223</t>
+          <t>MB6266</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2415,12 +2383,12 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Historical 2025 draw only; season dates not validated in current DATABASE</t>
+          <t>Contact Operator for 2026 season dates</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -2430,14 +2398,10 @@
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>CROSSWALK_CONFIRMED_ACTIVE_SAME_CODE_IN_2025_PDF</t>
-        </is>
-      </c>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="3" t="inlineStr">
         <is>
           <t>2025</t>
@@ -2451,962 +2415,12 @@
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>5.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="28" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Two Bear CWMU</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>MB6224</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>Moose</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>Any Legal Weapon</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>CWMU</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>Historical 2025 draw only; season dates not validated in current DATABASE</t>
-        </is>
-      </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J29" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t>CROSSWALK_CONFIRMED_ACTIVE_SAME_CODE_IN_2025_PDF</t>
-        </is>
-      </c>
-      <c r="L29" s="5" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="M29" s="5" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="N29" s="5" t="inlineStr"/>
-      <c r="O29" s="5" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="28" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Wallsburg CWMU</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>MB6225</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Moose</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Any Legal Weapon</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>CWMU</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>Contact operator for season dates</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J30" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>OIL_2025_PDF_AND_HARVEST_CONFIRMED_ACTIVE_CWMU_REVIEWED</t>
-        </is>
-      </c>
-      <c r="L30" s="3" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="M30" s="3" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="N30" s="3" t="inlineStr"/>
-      <c r="O30" s="3" t="inlineStr">
-        <is>
           <t>4.0</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Chimney Rock CWMU</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>MB6240</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>Moose</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>Any Legal Weapon</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>CWMU</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>Historical 2025 draw only; season dates not validated in current DATABASE</t>
-        </is>
-      </c>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J31" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K31" s="4" t="inlineStr">
-        <is>
-          <t>CROSSWALK_CONFIRMED_ACTIVE_SAME_CODE_IN_2025_PDF</t>
-        </is>
-      </c>
-      <c r="L31" s="5" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="M31" s="5" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="N31" s="5" t="inlineStr"/>
-      <c r="O31" s="5" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Hardscrabble CWMU</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>MB6251</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Moose</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Any Legal Weapon</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>CWMU</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>Contact Operator for 2026 season dates</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I32" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J32" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="3" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="M32" s="3" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="N32" s="3" t="inlineStr"/>
-      <c r="O32" s="3" t="inlineStr">
-        <is>
-          <t>5.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>SJ Ranch CWMU</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>MB6254</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>Moose</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>Any Legal Weapon</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>CWMU</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>Historical 2025 draw only; season dates not validated in current DATABASE</t>
-        </is>
-      </c>
-      <c r="H33" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I33" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J33" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K33" s="4" t="inlineStr">
-        <is>
-          <t>CROSSWALK_CONFIRMED_ACTIVE_SAME_CODE_IN_2025_PDF</t>
-        </is>
-      </c>
-      <c r="L33" s="5" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="M33" s="5" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="N33" s="5" t="inlineStr"/>
-      <c r="O33" s="5" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Woodruff Creek South CWMU</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>MB6256</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Moose</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Any Legal Weapon</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>CWMU</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>Contact Operator for 2026 season dates</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr"/>
-      <c r="L34" s="3" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="M34" s="3" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="N34" s="3" t="inlineStr"/>
-      <c r="O34" s="3" t="inlineStr">
-        <is>
-          <t>4.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="28" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>Ingham Peak CWMU</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>MB6257</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>Moose</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>Any Legal Weapon</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>CWMU</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>Contact operator for season dates</t>
-        </is>
-      </c>
-      <c r="H35" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I35" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J35" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K35" s="4" t="inlineStr">
-        <is>
-          <t>OIL_2025_PDF_AND_HARVEST_CONFIRMED_ACTIVE_CWMU_REVIEWED</t>
-        </is>
-      </c>
-      <c r="L35" s="5" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="M35" s="5" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="N35" s="5" t="inlineStr"/>
-      <c r="O35" s="5" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="28" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Jacob's Creek CWMU</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>MB6258</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>Moose</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Any Legal Weapon</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>CWMU</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>Contact Operator for 2026 season dates</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I36" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J36" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr"/>
-      <c r="L36" s="3" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="M36" s="3" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="N36" s="3" t="inlineStr"/>
-      <c r="O36" s="3" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="28" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>Royal Ivory Outfitters CWMU</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>MB6259</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>Moose</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>Any Legal Weapon</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>CWMU</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>Historical 2025 draw only; season dates not validated in current DATABASE</t>
-        </is>
-      </c>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I37" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J37" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K37" s="4" t="inlineStr">
-        <is>
-          <t>CROSSWALK_CONFIRMED_ACTIVE_SAME_CODE_IN_2025_PDF</t>
-        </is>
-      </c>
-      <c r="L37" s="5" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="M37" s="5" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="N37" s="5" t="inlineStr"/>
-      <c r="O37" s="5" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Junction Valley CWMU</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>MB6262</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>Moose</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Any Legal Weapon</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>CWMU</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Contact Operator for 2026 season dates</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I38" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J38" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K38" s="2" t="inlineStr"/>
-      <c r="L38" s="3" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="M38" s="3" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="N38" s="3" t="inlineStr"/>
-      <c r="O38" s="3" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="28" customHeight="1">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>Moon Ranch CWMU</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>MB6263</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>Moose</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>Any Legal Weapon</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>CWMU</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr">
-        <is>
-          <t>Historical 2025 draw only; season dates not validated in current DATABASE</t>
-        </is>
-      </c>
-      <c r="H39" s="5" t="inlineStr"/>
-      <c r="I39" s="5" t="inlineStr"/>
-      <c r="J39" s="5" t="inlineStr"/>
-      <c r="K39" s="4" t="inlineStr">
-        <is>
-          <t>HISTORICAL_2025_DRAW_ONLY_NOT_ACTIVE_2026</t>
-        </is>
-      </c>
-      <c r="L39" s="5" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="M39" s="5" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="N39" s="5" t="inlineStr"/>
-      <c r="O39" s="5" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="28" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Sand Creek CWMU</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>MB6264</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>Moose</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Any Legal Weapon</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>CWMU</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>Historical 2025 draw only; season dates not validated in current DATABASE</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr"/>
-      <c r="I40" s="3" t="inlineStr"/>
-      <c r="J40" s="3" t="inlineStr"/>
-      <c r="K40" s="2" t="inlineStr">
-        <is>
-          <t>HISTORICAL_2025_DRAW_ONLY_NOT_ACTIVE_2026</t>
-        </is>
-      </c>
-      <c r="L40" s="3" t="inlineStr"/>
-      <c r="M40" s="3" t="inlineStr"/>
-      <c r="N40" s="3" t="inlineStr"/>
-      <c r="O40" s="3" t="inlineStr"/>
-    </row>
-    <row r="41" ht="28" customHeight="1">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>Little Pole Canyon CWMU</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>MB6265</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>Moose</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>Any Legal Weapon</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>CWMU</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>Contact Operator for 2026 season dates</t>
-        </is>
-      </c>
-      <c r="H41" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I41" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J41" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K41" s="4" t="inlineStr"/>
-      <c r="L41" s="5" t="inlineStr"/>
-      <c r="M41" s="5" t="inlineStr"/>
-      <c r="N41" s="5" t="inlineStr"/>
-      <c r="O41" s="5" t="inlineStr"/>
-    </row>
-    <row r="42" ht="28" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Weber Florence Creek/Stillman Creek CWMU</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>MB6266</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Moose</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Any Legal Weapon</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>CWMU</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>Contact Operator for 2026 season dates</t>
-        </is>
-      </c>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I42" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J42" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr"/>
-      <c r="L42" s="3" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="M42" s="3" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="N42" s="3" t="inlineStr"/>
-      <c r="O42" s="3" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O42"/>
+  <autoFilter ref="A1:O28"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.15" right="0.15" top="0.25" bottom="0.25" header="0.1" footer="0.1"/>
   <pageSetup orientation="landscape" paperSize="5" fitToHeight="0" fitToWidth="1"/>

</xml_diff>